<commit_message>
Se termina BackEnd de egresos comprometido del capítulo 4
</commit_message>
<xml_diff>
--- a/public/Guia/4000-DevengadoFaltantes-CuentasConceptos.xlsx
+++ b/public/Guia/4000-DevengadoFaltantes-CuentasConceptos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\Guia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA3C626-9DF8-4FDC-9004-F12372C3474C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA154B3-AE19-45EC-AD86-83C76B5863D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="12">
   <si>
     <t>Presupuestal - Cargo</t>
   </si>
@@ -60,6 +60,18 @@
   </si>
   <si>
     <t>Por el devengado por Pensiones y Jubilaciones</t>
+  </si>
+  <si>
+    <t>cuenta</t>
+  </si>
+  <si>
+    <t>clasificador</t>
+  </si>
+  <si>
+    <t>concepto</t>
+  </si>
+  <si>
+    <t>tipo</t>
   </si>
 </sst>
 </file>
@@ -444,22 +456,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>6</v>
@@ -468,12 +480,12 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -482,12 +494,12 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
@@ -496,12 +508,12 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>6</v>
@@ -510,12 +522,12 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
@@ -524,13 +536,22 @@
         <v>7</v>
       </c>
       <c r="D6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>

</xml_diff>